<commit_message>
Added comments for the Scrolly Telling files
</commit_message>
<xml_diff>
--- a/Slow Reveal Recreations/anti-lynching-bill-map/text_position.xlsx
+++ b/Slow Reveal Recreations/anti-lynching-bill-map/text_position.xlsx
@@ -1,31 +1,43 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gvsu365-my.sharepoint.com/personal/s_cousilou_gvsu_edu/Documents/GVSU/Work/R Files/slow-reveal-graphs/Slow Reveal Recreations/anti-lynching-bill-map/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1070" documentId="11_F25DC773A252ABDACC10485159997CA65BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0CEEED29-887E-422B-84DD-E0B8C98ED4DB}"/>
+  <xr:revisionPtr revIDLastSave="1445" documentId="11_F25DC773A252ABDACC10485159997CA65BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE15901E-103B-4B5A-9D37-824BF914DB3D}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Horizontal Text" sheetId="1" r:id="rId1"/>
+    <sheet name="State" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="220">
   <si>
     <t>y</t>
   </si>
@@ -249,9 +261,6 @@
     <t>&lt;span style='color:red;'&gt;7&lt;/span&gt;</t>
   </si>
   <si>
-    <t>&lt;span style='color:black;'&gt;326&lt;/span&gt;</t>
-  </si>
-  <si>
     <t>&lt;span style='color:red;'&gt;1&lt;/span&gt;&lt;span style='color:black;'&gt; - 1&lt;/span&gt;</t>
   </si>
   <si>
@@ -376,6 +385,318 @@
   </si>
   <si>
     <t>&lt;span style='color:red;'&gt;80&lt;/span&gt;&lt;span style='color:#FCF2DA;'&gt; -&lt;/span&gt;</t>
+  </si>
+  <si>
+    <t>x_adj</t>
+  </si>
+  <si>
+    <t>&lt;span style='color:red;'&gt;405&lt;/span&gt;&lt;span style='color:#FCF2DA;'&gt; -&lt;/span&gt;</t>
+  </si>
+  <si>
+    <t>&lt;span style='color:red;'&gt;405&lt;/span&gt;&lt;span style='color:black;'&gt; -&lt;/span&gt;</t>
+  </si>
+  <si>
+    <t>size</t>
+  </si>
+  <si>
+    <t>&lt;span style='color:red;'&gt;326&lt;/span&gt;</t>
+  </si>
+  <si>
+    <t>alabama</t>
+  </si>
+  <si>
+    <t>ALA.</t>
+  </si>
+  <si>
+    <t>arizona</t>
+  </si>
+  <si>
+    <t>ARIZ.</t>
+  </si>
+  <si>
+    <t>arkansas</t>
+  </si>
+  <si>
+    <t>ARK.</t>
+  </si>
+  <si>
+    <t>california</t>
+  </si>
+  <si>
+    <t>CALIF.</t>
+  </si>
+  <si>
+    <t>colorado</t>
+  </si>
+  <si>
+    <t>COLO.</t>
+  </si>
+  <si>
+    <t>connecticut</t>
+  </si>
+  <si>
+    <t>C.T.</t>
+  </si>
+  <si>
+    <t>delaware</t>
+  </si>
+  <si>
+    <t>DEL.</t>
+  </si>
+  <si>
+    <t>florida</t>
+  </si>
+  <si>
+    <t>FLA.</t>
+  </si>
+  <si>
+    <t>georgia</t>
+  </si>
+  <si>
+    <t>GA.</t>
+  </si>
+  <si>
+    <t>idaho</t>
+  </si>
+  <si>
+    <t>IDAHO</t>
+  </si>
+  <si>
+    <t>illinois</t>
+  </si>
+  <si>
+    <t>ILL.</t>
+  </si>
+  <si>
+    <t>indiana</t>
+  </si>
+  <si>
+    <t>IND.</t>
+  </si>
+  <si>
+    <t>iowa</t>
+  </si>
+  <si>
+    <t>IOWA</t>
+  </si>
+  <si>
+    <t>kansas</t>
+  </si>
+  <si>
+    <t>KANS.</t>
+  </si>
+  <si>
+    <t>kentucky</t>
+  </si>
+  <si>
+    <t>KY.</t>
+  </si>
+  <si>
+    <t>louisiana</t>
+  </si>
+  <si>
+    <t>LA.</t>
+  </si>
+  <si>
+    <t>maine</t>
+  </si>
+  <si>
+    <t>MAINE</t>
+  </si>
+  <si>
+    <t>maryland</t>
+  </si>
+  <si>
+    <t>MD.</t>
+  </si>
+  <si>
+    <t>massachusetts</t>
+  </si>
+  <si>
+    <t>MASS.</t>
+  </si>
+  <si>
+    <t>michigan</t>
+  </si>
+  <si>
+    <t>MICH.</t>
+  </si>
+  <si>
+    <t>minnesota</t>
+  </si>
+  <si>
+    <t>MINN.</t>
+  </si>
+  <si>
+    <t>mississippi</t>
+  </si>
+  <si>
+    <t>MISS.</t>
+  </si>
+  <si>
+    <t>missouri</t>
+  </si>
+  <si>
+    <t>MO.</t>
+  </si>
+  <si>
+    <t>montana</t>
+  </si>
+  <si>
+    <t>MONT.</t>
+  </si>
+  <si>
+    <t>nebraska</t>
+  </si>
+  <si>
+    <t>NEBR.</t>
+  </si>
+  <si>
+    <t>nevada</t>
+  </si>
+  <si>
+    <t>NEV.</t>
+  </si>
+  <si>
+    <t>new hampshire</t>
+  </si>
+  <si>
+    <t>N.H.</t>
+  </si>
+  <si>
+    <t>new jersey</t>
+  </si>
+  <si>
+    <t>N.J.</t>
+  </si>
+  <si>
+    <t>new mexico</t>
+  </si>
+  <si>
+    <t>N.MEX.</t>
+  </si>
+  <si>
+    <t>new york</t>
+  </si>
+  <si>
+    <t>N.Y</t>
+  </si>
+  <si>
+    <t>north carolina</t>
+  </si>
+  <si>
+    <t>N.C.</t>
+  </si>
+  <si>
+    <t>north dakota</t>
+  </si>
+  <si>
+    <t>N.DAK.</t>
+  </si>
+  <si>
+    <t>ohio</t>
+  </si>
+  <si>
+    <t>OHIO</t>
+  </si>
+  <si>
+    <t>oklahoma</t>
+  </si>
+  <si>
+    <t>OKLA.</t>
+  </si>
+  <si>
+    <t>oregon</t>
+  </si>
+  <si>
+    <t>OREG.</t>
+  </si>
+  <si>
+    <t>pennsylvania</t>
+  </si>
+  <si>
+    <t>PA.</t>
+  </si>
+  <si>
+    <t>rhode island</t>
+  </si>
+  <si>
+    <t>R.I.</t>
+  </si>
+  <si>
+    <t>south carolina</t>
+  </si>
+  <si>
+    <t>S.C.</t>
+  </si>
+  <si>
+    <t>south dakota</t>
+  </si>
+  <si>
+    <t>S.DAK.</t>
+  </si>
+  <si>
+    <t>tennessee</t>
+  </si>
+  <si>
+    <t>TENN.</t>
+  </si>
+  <si>
+    <t>texas</t>
+  </si>
+  <si>
+    <t>TEXAS</t>
+  </si>
+  <si>
+    <t>utah</t>
+  </si>
+  <si>
+    <t>UTAH</t>
+  </si>
+  <si>
+    <t>vermont</t>
+  </si>
+  <si>
+    <t>VT.</t>
+  </si>
+  <si>
+    <t>virginia</t>
+  </si>
+  <si>
+    <t>VA.</t>
+  </si>
+  <si>
+    <t>washington</t>
+  </si>
+  <si>
+    <t>WASH.</t>
+  </si>
+  <si>
+    <t>west virginia</t>
+  </si>
+  <si>
+    <t>W.VA.</t>
+  </si>
+  <si>
+    <t>wisconsin</t>
+  </si>
+  <si>
+    <t>WIS.</t>
+  </si>
+  <si>
+    <t>wyoming</t>
+  </si>
+  <si>
+    <t>WYO.</t>
+  </si>
+  <si>
+    <t>region</t>
+  </si>
+  <si>
+    <t>Abb</t>
+  </si>
+  <si>
+    <t>angle</t>
   </si>
 </sst>
 </file>
@@ -697,7 +1018,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E87"/>
+  <dimension ref="A1:I87"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="11.7109375" bestFit="1" customWidth="1"/>
@@ -705,7 +1026,7 @@
     <col min="4" max="4" width="62.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -719,35 +1040,54 @@
         <v>1</v>
       </c>
       <c r="E1" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+        <v>101</v>
+      </c>
+      <c r="F1" t="s">
+        <v>116</v>
+      </c>
+      <c r="G1" t="s">
+        <v>119</v>
+      </c>
+      <c r="H1" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2">
-        <v>-87.551620999999997</v>
+        <v>-87.051620999999997</v>
       </c>
       <c r="C2">
-        <v>34.467106000000001</v>
+        <v>34.217106000000001</v>
       </c>
       <c r="D2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F2">
+        <f>B2+0.5</f>
+        <v>-86.551620999999997</v>
+      </c>
+      <c r="G2">
+        <v>16</v>
+      </c>
+      <c r="H2">
+        <v>6.4829999999999997</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
       <c r="B3">
-        <v>-87.551620999999997</v>
+        <v>-87.051620999999997</v>
       </c>
       <c r="C3">
-        <v>34.467106000000001</v>
+        <v>34.217106000000001</v>
       </c>
       <c r="D3" t="s">
         <v>46</v>
@@ -755,16 +1095,26 @@
       <c r="E3">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F3">
+        <f t="shared" ref="F3:F66" si="0">B3+0.5</f>
+        <v>-86.551620999999997</v>
+      </c>
+      <c r="G3">
+        <v>16</v>
+      </c>
+      <c r="H3">
+        <v>6.4829999999999997</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
       <c r="B4">
-        <v>-86.314418000000003</v>
+        <v>-85.814418000000003</v>
       </c>
       <c r="C4">
-        <v>33.709789999999998</v>
+        <v>33.459789999999998</v>
       </c>
       <c r="D4" t="s">
         <v>50</v>
@@ -772,30 +1122,50 @@
       <c r="E4">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F4">
+        <f t="shared" si="0"/>
+        <v>-85.314418000000003</v>
+      </c>
+      <c r="G4">
+        <v>16</v>
+      </c>
+      <c r="H4">
+        <v>6.4829999999999997</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
       <c r="B5">
-        <v>-112.58563100000001</v>
+        <v>-112.08563100000001</v>
       </c>
       <c r="C5">
         <v>36.310676999999998</v>
       </c>
       <c r="D5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E5">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F5">
+        <f t="shared" si="0"/>
+        <v>-111.58563100000001</v>
+      </c>
+      <c r="G5">
+        <v>16</v>
+      </c>
+      <c r="H5">
+        <v>-8.0429999999999993</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
       <c r="B6">
-        <v>-112.58563100000001</v>
+        <v>-112.08563100000001</v>
       </c>
       <c r="C6">
         <v>36.310676999999998</v>
@@ -806,16 +1176,26 @@
       <c r="E6">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F6">
+        <f t="shared" si="0"/>
+        <v>-111.58563100000001</v>
+      </c>
+      <c r="G6">
+        <v>16</v>
+      </c>
+      <c r="H6">
+        <v>-8.0429999999999993</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
       <c r="B7">
-        <v>-112.58563100000001</v>
+        <v>-112.08563100000001</v>
       </c>
       <c r="C7">
-        <v>33.456319000000001</v>
+        <v>32.956319000000001</v>
       </c>
       <c r="D7" t="s">
         <v>52</v>
@@ -823,8 +1203,18 @@
       <c r="E7">
         <v>2</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F7">
+        <f t="shared" si="0"/>
+        <v>-111.58563100000001</v>
+      </c>
+      <c r="G7">
+        <v>16</v>
+      </c>
+      <c r="H7">
+        <v>-4.9340000000000002</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -840,8 +1230,18 @@
       <c r="E8">
         <v>2</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F8">
+        <f t="shared" si="0"/>
+        <v>-92.053292999999996</v>
+      </c>
+      <c r="G8">
+        <v>16</v>
+      </c>
+      <c r="H8">
+        <v>2.6259999999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -857,30 +1257,50 @@
       <c r="E9">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F9">
+        <f t="shared" si="0"/>
+        <v>-91.985444000000001</v>
+      </c>
+      <c r="G9">
+        <v>16</v>
+      </c>
+      <c r="H9">
+        <v>2.6259999999999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>6</v>
       </c>
       <c r="B10">
-        <v>-122.782814</v>
+        <v>-122.282814</v>
       </c>
       <c r="C10">
         <v>40.873595999999999</v>
       </c>
       <c r="D10" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E10">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F10">
+        <f t="shared" si="0"/>
+        <v>-121.782814</v>
+      </c>
+      <c r="G10">
+        <v>16</v>
+      </c>
+      <c r="H10">
+        <v>-17.904</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>6</v>
       </c>
       <c r="B11">
-        <v>-122.782814</v>
+        <v>-122.282814</v>
       </c>
       <c r="C11">
         <v>40.873595999999999</v>
@@ -891,16 +1311,26 @@
       <c r="E11">
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F11">
+        <f t="shared" si="0"/>
+        <v>-121.782814</v>
+      </c>
+      <c r="G11">
+        <v>16</v>
+      </c>
+      <c r="H11">
+        <v>-17.904</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>6</v>
       </c>
       <c r="B12">
-        <v>-118.61556</v>
+        <v>-118.86556</v>
       </c>
       <c r="C12">
-        <v>35.571786000000003</v>
+        <v>35.821786000000003</v>
       </c>
       <c r="D12" t="s">
         <v>55</v>
@@ -908,8 +1338,18 @@
       <c r="E12">
         <v>2</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F12">
+        <f t="shared" si="0"/>
+        <v>-118.36556</v>
+      </c>
+      <c r="G12">
+        <v>16</v>
+      </c>
+      <c r="H12">
+        <v>-3.048</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>6</v>
       </c>
@@ -917,7 +1357,7 @@
         <v>-118.11556</v>
       </c>
       <c r="C13">
-        <v>35.07179</v>
+        <v>35.321786000000003</v>
       </c>
       <c r="D13" t="s">
         <v>56</v>
@@ -925,8 +1365,18 @@
       <c r="E13">
         <v>2</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F13">
+        <f t="shared" si="0"/>
+        <v>-117.61556</v>
+      </c>
+      <c r="G13">
+        <v>16</v>
+      </c>
+      <c r="H13">
+        <v>-0.79600000000000004</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>6</v>
       </c>
@@ -934,7 +1384,7 @@
         <v>-117.61556</v>
       </c>
       <c r="C14">
-        <v>34.571786000000003</v>
+        <v>34.821786000000003</v>
       </c>
       <c r="D14" t="s">
         <v>57</v>
@@ -942,16 +1392,26 @@
       <c r="E14">
         <v>2</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F14">
+        <f t="shared" si="0"/>
+        <v>-117.11556</v>
+      </c>
+      <c r="G14">
+        <v>16</v>
+      </c>
+      <c r="H14">
+        <v>-1.2729999999999999</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>6</v>
       </c>
       <c r="B15">
-        <v>-117.11556</v>
+        <v>-116.61556</v>
       </c>
       <c r="C15">
-        <v>34.07179</v>
+        <v>34.321786000000003</v>
       </c>
       <c r="D15" t="s">
         <v>58</v>
@@ -959,16 +1419,26 @@
       <c r="E15">
         <v>2</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F15">
+        <f t="shared" si="0"/>
+        <v>-116.11556</v>
+      </c>
+      <c r="G15">
+        <v>16</v>
+      </c>
+      <c r="H15">
+        <v>-1.5069999999999999</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>6</v>
       </c>
       <c r="B16">
-        <v>-116.61556</v>
+        <v>-116.11556</v>
       </c>
       <c r="C16">
-        <v>33.571786000000003</v>
+        <v>33.821786000000003</v>
       </c>
       <c r="D16" t="s">
         <v>59</v>
@@ -976,13 +1446,23 @@
       <c r="E16">
         <v>2</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F16">
+        <f t="shared" si="0"/>
+        <v>-115.61556</v>
+      </c>
+      <c r="G16">
+        <v>16</v>
+      </c>
+      <c r="H16">
+        <v>1.123</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>7</v>
       </c>
       <c r="B17">
-        <v>-106.319619</v>
+        <v>-105.819619</v>
       </c>
       <c r="C17">
         <v>39.9803</v>
@@ -993,33 +1473,53 @@
       <c r="E17">
         <v>2</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F17">
+        <f t="shared" si="0"/>
+        <v>-105.319619</v>
+      </c>
+      <c r="G17">
+        <v>16</v>
+      </c>
+      <c r="H17">
+        <v>-4.5570000000000004</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>8</v>
       </c>
       <c r="B18">
-        <v>-82.917704000000001</v>
+        <v>-82.417704000000001</v>
       </c>
       <c r="C18">
-        <v>30.132432999999999</v>
+        <v>29.882432999999999</v>
       </c>
       <c r="D18" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E18">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F18">
+        <f t="shared" si="0"/>
+        <v>-81.917704000000001</v>
+      </c>
+      <c r="G18">
+        <v>16</v>
+      </c>
+      <c r="H18">
+        <v>-1.736</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>8</v>
       </c>
       <c r="B19">
-        <v>-82.917704000000001</v>
+        <v>-82.417704000000001</v>
       </c>
       <c r="C19">
-        <v>30.132432999999999</v>
+        <v>29.882432999999999</v>
       </c>
       <c r="D19" t="s">
         <v>47</v>
@@ -1027,16 +1527,26 @@
       <c r="E19">
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F19">
+        <f t="shared" si="0"/>
+        <v>-81.917704000000001</v>
+      </c>
+      <c r="G19">
+        <v>16</v>
+      </c>
+      <c r="H19">
+        <v>-1.736</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>8</v>
       </c>
       <c r="B20">
-        <v>-82.218414999999993</v>
+        <v>-81.718414999999993</v>
       </c>
       <c r="C20">
-        <v>29.408714</v>
+        <v>29.158714</v>
       </c>
       <c r="D20" t="s">
         <v>61</v>
@@ -1044,33 +1554,53 @@
       <c r="E20">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F20">
+        <f t="shared" si="0"/>
+        <v>-81.218414999999993</v>
+      </c>
+      <c r="G20">
+        <v>16</v>
+      </c>
+      <c r="H20">
+        <v>-1.736</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>9</v>
       </c>
       <c r="B21">
-        <v>-84.646884999999997</v>
+        <v>-84.146884999999997</v>
       </c>
       <c r="C21">
-        <v>34.533602000000002</v>
+        <v>34.283602000000002</v>
       </c>
       <c r="D21" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E21">
         <v>0</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F21">
+        <f t="shared" si="0"/>
+        <v>-83.646884999999997</v>
+      </c>
+      <c r="G21">
+        <v>16</v>
+      </c>
+      <c r="H21">
+        <v>6.3840000000000003</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>9</v>
       </c>
       <c r="B22">
-        <v>-84.646884999999997</v>
+        <v>-84.146884999999997</v>
       </c>
       <c r="C22">
-        <v>34.533602000000002</v>
+        <v>34.283602000000002</v>
       </c>
       <c r="D22" t="s">
         <v>48</v>
@@ -1078,16 +1608,26 @@
       <c r="E22">
         <v>1</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F22">
+        <f t="shared" si="0"/>
+        <v>-83.646884999999997</v>
+      </c>
+      <c r="G22">
+        <v>16</v>
+      </c>
+      <c r="H22">
+        <v>6.3840000000000003</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>9</v>
       </c>
       <c r="B23">
-        <v>-83.624848</v>
+        <v>-83.124848</v>
       </c>
       <c r="C23">
-        <v>33.866261000000002</v>
+        <v>33.616261000000002</v>
       </c>
       <c r="D23" t="s">
         <v>62</v>
@@ -1095,33 +1635,53 @@
       <c r="E23">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F23">
+        <f t="shared" si="0"/>
+        <v>-82.624848</v>
+      </c>
+      <c r="G23">
+        <v>16</v>
+      </c>
+      <c r="H23">
+        <v>6.3840000000000003</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>10</v>
       </c>
       <c r="B24">
-        <v>-116.098294</v>
+        <v>-115.348294</v>
       </c>
       <c r="C24">
-        <v>45.037768999999997</v>
+        <v>44.787768999999997</v>
       </c>
       <c r="D24" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E24">
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F24">
+        <f t="shared" si="0"/>
+        <v>-114.848294</v>
+      </c>
+      <c r="G24">
+        <v>16</v>
+      </c>
+      <c r="H24">
+        <v>-10.305</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>10</v>
       </c>
       <c r="B25">
-        <v>-116.098294</v>
+        <v>-115.348294</v>
       </c>
       <c r="C25">
-        <v>45.037768999999997</v>
+        <v>44.787768999999997</v>
       </c>
       <c r="D25" t="s">
         <v>69</v>
@@ -1129,13 +1689,23 @@
       <c r="E25">
         <v>1</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F25">
+        <f t="shared" si="0"/>
+        <v>-114.848294</v>
+      </c>
+      <c r="G25">
+        <v>16</v>
+      </c>
+      <c r="H25">
+        <v>-10.305</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>10</v>
       </c>
       <c r="B26">
-        <v>-114.47823200000001</v>
+        <v>-113.97823200000001</v>
       </c>
       <c r="C26">
         <v>42.740774000000002</v>
@@ -1146,13 +1716,23 @@
       <c r="E26">
         <v>2</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F26">
+        <f t="shared" si="0"/>
+        <v>-113.47823200000001</v>
+      </c>
+      <c r="G26">
+        <v>16</v>
+      </c>
+      <c r="H26">
+        <v>-6.9870000000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>11</v>
       </c>
       <c r="B27">
-        <v>-89.370014999999995</v>
+        <v>-88.870014999999995</v>
       </c>
       <c r="C27">
         <v>41.121966</v>
@@ -1163,13 +1743,23 @@
       <c r="E27">
         <v>2</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F27">
+        <f t="shared" si="0"/>
+        <v>-88.370014999999995</v>
+      </c>
+      <c r="G27">
+        <v>16</v>
+      </c>
+      <c r="H27">
+        <v>0.92400000000000004</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>12</v>
       </c>
       <c r="B28">
-        <v>-86.393799000000001</v>
+        <v>-85.893799000000001</v>
       </c>
       <c r="C28">
         <v>41.174652000000002</v>
@@ -1180,13 +1770,23 @@
       <c r="E28">
         <v>2</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F28">
+        <f t="shared" si="0"/>
+        <v>-85.393799000000001</v>
+      </c>
+      <c r="G28">
+        <v>16</v>
+      </c>
+      <c r="H28">
+        <v>0.92400000000000004</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>13</v>
       </c>
       <c r="B29">
-        <v>-94.411345999999995</v>
+        <v>-93.911345999999995</v>
       </c>
       <c r="C29">
         <v>42.792228999999999</v>
@@ -1197,13 +1797,23 @@
       <c r="E29">
         <v>2</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F29">
+        <f t="shared" si="0"/>
+        <v>-93.411345999999995</v>
+      </c>
+      <c r="G29">
+        <v>16</v>
+      </c>
+      <c r="H29">
+        <v>0.92400000000000004</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>14</v>
       </c>
       <c r="B30">
-        <v>-98.956721000000002</v>
+        <v>-98.456721000000002</v>
       </c>
       <c r="C30">
         <v>39.263188</v>
@@ -1214,33 +1824,53 @@
       <c r="E30">
         <v>2</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F30">
+        <f t="shared" si="0"/>
+        <v>-97.956721000000002</v>
+      </c>
+      <c r="G30">
+        <v>16</v>
+      </c>
+      <c r="H30">
+        <v>-1.54</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>15</v>
       </c>
       <c r="B31">
-        <v>-84.494012999999995</v>
+        <v>-83.994012999999995</v>
       </c>
       <c r="C31">
-        <v>38.252592999999997</v>
+        <v>38.002592999999997</v>
       </c>
       <c r="D31" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E31">
         <v>0</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F31">
+        <f t="shared" si="0"/>
+        <v>-83.494012999999995</v>
+      </c>
+      <c r="G31">
+        <v>16</v>
+      </c>
+      <c r="H31">
+        <v>2.7050000000000001</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>15</v>
       </c>
       <c r="B32">
-        <v>-84.494012999999995</v>
+        <v>-83.994012999999995</v>
       </c>
       <c r="C32">
-        <v>38.252592999999997</v>
+        <v>38.002592999999997</v>
       </c>
       <c r="D32" t="s">
         <v>49</v>
@@ -1248,8 +1878,18 @@
       <c r="E32">
         <v>1</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F32">
+        <f t="shared" si="0"/>
+        <v>-83.494012999999995</v>
+      </c>
+      <c r="G32">
+        <v>16</v>
+      </c>
+      <c r="H32">
+        <v>2.7050000000000001</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>15</v>
       </c>
@@ -1257,7 +1897,7 @@
         <v>-83.272722000000002</v>
       </c>
       <c r="C33">
-        <v>37.574567000000002</v>
+        <v>37.074567000000002</v>
       </c>
       <c r="D33" t="s">
         <v>71</v>
@@ -1265,30 +1905,50 @@
       <c r="E33">
         <v>1</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F33">
+        <f t="shared" si="0"/>
+        <v>-82.772722000000002</v>
+      </c>
+      <c r="G33">
+        <v>16</v>
+      </c>
+      <c r="H33">
+        <v>2.7050000000000001</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>16</v>
       </c>
       <c r="B34">
-        <v>-92.89819</v>
+        <v>-92.39819</v>
       </c>
       <c r="C34">
         <v>32.215719999999997</v>
       </c>
       <c r="D34" t="s">
-        <v>74</v>
+        <v>120</v>
       </c>
       <c r="E34">
         <v>2</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F34">
+        <f t="shared" si="0"/>
+        <v>-91.89819</v>
+      </c>
+      <c r="G34">
+        <v>16</v>
+      </c>
+      <c r="H34">
+        <v>0.39500000000000002</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>16</v>
       </c>
       <c r="B35">
-        <v>-92.739874</v>
+        <v>-92.239874</v>
       </c>
       <c r="C35">
         <v>30.457964</v>
@@ -1299,42 +1959,72 @@
       <c r="E35">
         <v>1</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F35">
+        <f t="shared" si="0"/>
+        <v>-91.739874</v>
+      </c>
+      <c r="G35">
+        <v>16</v>
+      </c>
+      <c r="H35">
+        <v>0.39500000000000002</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>17</v>
       </c>
       <c r="B36">
-        <v>-69.685015000000007</v>
+        <v>-68.975014999999999</v>
       </c>
       <c r="C36">
         <v>46.504477000000001</v>
       </c>
       <c r="D36" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E36">
         <v>0</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F36">
+        <f t="shared" si="0"/>
+        <v>-68.475014999999999</v>
+      </c>
+      <c r="G36">
+        <v>10</v>
+      </c>
+      <c r="H36">
+        <v>5.7679999999999998</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>17</v>
       </c>
       <c r="B37">
-        <v>-69.685015000000007</v>
+        <v>-68.975014999999999</v>
       </c>
       <c r="C37">
         <v>46.504477000000001</v>
       </c>
       <c r="D37" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E37">
         <v>1</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F37">
+        <f t="shared" si="0"/>
+        <v>-68.475014999999999</v>
+      </c>
+      <c r="G37">
+        <v>10</v>
+      </c>
+      <c r="H37">
+        <v>5.7679999999999998</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>17</v>
       </c>
@@ -1350,47 +2040,80 @@
       <c r="E38">
         <v>2</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F38">
+        <f t="shared" si="0"/>
+        <v>-69.615347</v>
+      </c>
+      <c r="G38">
+        <v>10</v>
+      </c>
+      <c r="H38">
+        <v>16.242999999999999</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>18</v>
       </c>
       <c r="B39">
-        <v>-76.394461000000007</v>
+        <v>-76.644461000000007</v>
       </c>
       <c r="C39">
-        <v>39.580083000000002</v>
+        <v>39.130082999999999</v>
       </c>
       <c r="D39" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E39">
         <v>0</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F39">
+        <f t="shared" si="0"/>
+        <v>-76.144461000000007</v>
+      </c>
+      <c r="G39">
+        <v>8</v>
+      </c>
+      <c r="H39">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>18</v>
       </c>
       <c r="B40">
-        <v>-76.394461000000007</v>
+        <v>-76.644461000000007</v>
       </c>
       <c r="C40">
-        <v>39.580083000000002</v>
+        <v>39.130082999999999</v>
       </c>
       <c r="D40" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E40">
         <v>1</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F40">
+        <f t="shared" si="0"/>
+        <v>-76.144461000000007</v>
+      </c>
+      <c r="G40">
+        <v>8</v>
+      </c>
+      <c r="H40">
+        <v>15</v>
+      </c>
+      <c r="I40">
+        <v>8.5310000000000006</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>19</v>
       </c>
       <c r="B41">
-        <v>-69.337142</v>
+        <v>-68.837142</v>
       </c>
       <c r="C41">
         <v>42.429639999999999</v>
@@ -1401,47 +2124,77 @@
       <c r="E41">
         <v>2</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F41">
+        <f t="shared" si="0"/>
+        <v>-68.337142</v>
+      </c>
+      <c r="G41">
+        <v>16</v>
+      </c>
+      <c r="H41">
+        <v>10.954000000000001</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>20</v>
       </c>
       <c r="B42">
-        <v>-85.525210000000001</v>
+        <v>-85.025210000000001</v>
       </c>
       <c r="C42">
         <v>44.375965000000001</v>
       </c>
       <c r="D42" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E42">
         <v>0</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F42">
+        <f t="shared" si="0"/>
+        <v>-84.525210000000001</v>
+      </c>
+      <c r="G42">
+        <v>12</v>
+      </c>
+      <c r="H42">
+        <v>2.3140000000000001</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>20</v>
       </c>
       <c r="B43">
-        <v>-85.525210000000001</v>
+        <v>-85.025210000000001</v>
       </c>
       <c r="C43">
         <v>44.375965000000001</v>
       </c>
       <c r="D43" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E43">
         <v>1</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F43">
+        <f t="shared" si="0"/>
+        <v>-84.525210000000001</v>
+      </c>
+      <c r="G43">
+        <v>12</v>
+      </c>
+      <c r="H43">
+        <v>2.3140000000000001</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>20</v>
       </c>
       <c r="B44">
-        <v>-84.914563999999999</v>
+        <v>-84.664563999999999</v>
       </c>
       <c r="C44">
         <v>42.404001000000001</v>
@@ -1452,13 +2205,23 @@
       <c r="E44">
         <v>2</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F44">
+        <f t="shared" si="0"/>
+        <v>-84.164563999999999</v>
+      </c>
+      <c r="G44">
+        <v>12</v>
+      </c>
+      <c r="H44">
+        <v>8.07</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>21</v>
       </c>
       <c r="B45">
-        <v>-94.787886</v>
+        <v>-94.287886</v>
       </c>
       <c r="C45">
         <v>47.631867</v>
@@ -1469,475 +2232,755 @@
       <c r="E45">
         <v>2</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F45">
+        <f t="shared" si="0"/>
+        <v>-93.787886</v>
+      </c>
+      <c r="G45">
+        <v>16</v>
+      </c>
+      <c r="H45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>22</v>
       </c>
       <c r="B46">
-        <v>-89.622590000000002</v>
+        <v>-89.372590000000002</v>
       </c>
       <c r="C46">
-        <v>34.444929000000002</v>
+        <v>34.194929000000002</v>
       </c>
       <c r="D46" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="E46">
         <v>0</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F46">
+        <f t="shared" si="0"/>
+        <v>-88.872590000000002</v>
+      </c>
+      <c r="G46">
+        <v>16</v>
+      </c>
+      <c r="H46">
+        <v>3.7149999999999999</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>22</v>
       </c>
       <c r="B47">
-        <v>-89.622590000000002</v>
+        <v>-89.372590000000002</v>
       </c>
       <c r="C47">
-        <v>34.444929000000002</v>
+        <v>34.194929000000002</v>
       </c>
       <c r="D47" t="s">
-        <v>49</v>
+        <v>118</v>
       </c>
       <c r="E47">
         <v>1</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F47">
+        <f t="shared" si="0"/>
+        <v>-88.872590000000002</v>
+      </c>
+      <c r="G47">
+        <v>16</v>
+      </c>
+      <c r="H47">
+        <v>3.7149999999999999</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>22</v>
       </c>
       <c r="B48">
-        <v>-88.815719000000001</v>
+        <v>-88.872590000000002</v>
       </c>
       <c r="C48">
-        <v>33.955545000000001</v>
+        <v>33.555545000000002</v>
       </c>
       <c r="D48" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="E48">
         <v>1</v>
       </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F48">
+        <f t="shared" si="0"/>
+        <v>-88.372590000000002</v>
+      </c>
+      <c r="G48">
+        <v>16</v>
+      </c>
+      <c r="H48">
+        <v>3.7149999999999999</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>23</v>
       </c>
       <c r="B49">
-        <v>-93.797201000000001</v>
+        <v>-93.297201000000001</v>
       </c>
       <c r="C49">
         <v>39.841631999999997</v>
       </c>
       <c r="D49" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E49">
         <v>0</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F49">
+        <f t="shared" si="0"/>
+        <v>-92.797201000000001</v>
+      </c>
+      <c r="G49">
+        <v>16</v>
+      </c>
+      <c r="H49">
+        <v>4.0860000000000003</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>23</v>
       </c>
       <c r="B50">
-        <v>-93.797201000000001</v>
+        <v>-93.297201000000001</v>
       </c>
       <c r="C50">
         <v>39.841631999999997</v>
       </c>
       <c r="D50" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E50">
         <v>1</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F50">
+        <f t="shared" si="0"/>
+        <v>-92.797201000000001</v>
+      </c>
+      <c r="G50">
+        <v>16</v>
+      </c>
+      <c r="H50">
+        <v>4.0860000000000003</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>23</v>
       </c>
       <c r="B51">
-        <v>-92.394977999999995</v>
+        <v>-91.894977999999995</v>
       </c>
       <c r="C51">
         <v>37.583078999999998</v>
       </c>
       <c r="D51" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E51">
         <v>2</v>
       </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F51">
+        <f t="shared" si="0"/>
+        <v>-91.394977999999995</v>
+      </c>
+      <c r="G51">
+        <v>16</v>
+      </c>
+      <c r="H51">
+        <v>3.4340000000000002</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>24</v>
       </c>
       <c r="B52">
-        <v>-110.569141</v>
+        <v>-110.069141</v>
       </c>
       <c r="C52">
         <v>48.046407000000002</v>
       </c>
       <c r="D52" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E52">
         <v>2</v>
       </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F52">
+        <f t="shared" si="0"/>
+        <v>-109.569141</v>
+      </c>
+      <c r="G52">
+        <v>16</v>
+      </c>
+      <c r="H52">
+        <v>-3.4169999999999998</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>25</v>
       </c>
       <c r="B53">
-        <v>-100.51014600000001</v>
+        <v>-100.01014600000001</v>
       </c>
       <c r="C53">
         <v>42.328971000000003</v>
       </c>
       <c r="D53" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E53">
         <v>2</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F53">
+        <f t="shared" si="0"/>
+        <v>-99.510146000000006</v>
+      </c>
+      <c r="G53">
+        <v>16</v>
+      </c>
+      <c r="H53">
+        <v>-1.2729999999999999</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>26</v>
       </c>
       <c r="B54">
-        <v>-117.195756</v>
+        <v>-116.695756</v>
       </c>
       <c r="C54">
         <v>40.910656000000003</v>
       </c>
       <c r="D54" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E54">
         <v>2</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F54">
+        <f t="shared" si="0"/>
+        <v>-116.195756</v>
+      </c>
+      <c r="G54">
+        <v>16</v>
+      </c>
+      <c r="H54">
+        <v>-1.2729999999999999</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>27</v>
       </c>
       <c r="B55">
-        <v>-74.878185000000002</v>
+        <v>-74.628185000000002</v>
       </c>
       <c r="C55">
-        <v>39.858423000000002</v>
+        <v>39.608423000000002</v>
       </c>
       <c r="D55" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E55">
         <v>1</v>
       </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F55">
+        <f t="shared" si="0"/>
+        <v>-74.128185000000002</v>
+      </c>
+      <c r="G55">
+        <v>16</v>
+      </c>
+      <c r="H55">
+        <v>9.2110000000000003</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>27</v>
       </c>
       <c r="B56">
-        <v>-71.508325999999997</v>
+        <v>-71.008325999999997</v>
       </c>
       <c r="C56">
-        <v>40.152926999999998</v>
+        <v>39.652926999999998</v>
       </c>
       <c r="D56" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E56">
         <v>2</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F56">
+        <f t="shared" si="0"/>
+        <v>-70.508325999999997</v>
+      </c>
+      <c r="G56">
+        <v>16</v>
+      </c>
+      <c r="H56">
+        <v>8.093</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>27</v>
       </c>
       <c r="B57">
-        <v>-74.584170999999998</v>
+        <v>-74.334170999999998</v>
       </c>
       <c r="C57">
-        <v>40.806629000000001</v>
+        <v>40.556629000000001</v>
       </c>
       <c r="D57" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E57">
         <v>2</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F57">
+        <f t="shared" si="0"/>
+        <v>-73.834170999999998</v>
+      </c>
+      <c r="G57">
+        <v>16</v>
+      </c>
+      <c r="H57">
+        <v>9.2110000000000003</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>28</v>
       </c>
       <c r="B58">
-        <v>-106.91132399999999</v>
+        <v>-106.41132399999999</v>
       </c>
       <c r="C58">
         <v>35.909885000000003</v>
       </c>
       <c r="D58" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E58">
         <v>2</v>
       </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F58">
+        <f t="shared" si="0"/>
+        <v>-105.91132399999999</v>
+      </c>
+      <c r="G58">
+        <v>16</v>
+      </c>
+      <c r="H58">
+        <v>-3.4</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>29</v>
       </c>
       <c r="B59">
-        <v>-75.149583000000007</v>
+        <v>-74.649583000000007</v>
       </c>
       <c r="C59">
         <v>44.011690000000002</v>
       </c>
       <c r="D59" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E59">
         <v>2</v>
       </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F59">
+        <f t="shared" si="0"/>
+        <v>-74.149583000000007</v>
+      </c>
+      <c r="G59">
+        <v>16</v>
+      </c>
+      <c r="H59">
+        <v>-2.7726000000000002</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>30</v>
       </c>
       <c r="B60">
-        <v>-77.999262999999999</v>
+        <v>-77.499262999999999</v>
       </c>
       <c r="C60">
         <v>34.864491000000001</v>
       </c>
       <c r="D60" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E60">
         <v>1</v>
       </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F60">
+        <f t="shared" si="0"/>
+        <v>-76.999262999999999</v>
+      </c>
+      <c r="G60">
+        <v>16</v>
+      </c>
+      <c r="H60">
+        <v>6.5819999999999999</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>30</v>
       </c>
       <c r="B61">
-        <v>-77.727864999999994</v>
+        <v>-77.227864999999994</v>
       </c>
       <c r="C61">
         <v>35.952030999999998</v>
       </c>
       <c r="D61" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E61">
         <v>2</v>
       </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F61">
+        <f t="shared" si="0"/>
+        <v>-76.727864999999994</v>
+      </c>
+      <c r="G61">
+        <v>16</v>
+      </c>
+      <c r="H61">
+        <v>6.5819999999999999</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>31</v>
       </c>
       <c r="B62">
-        <v>-100.994269</v>
+        <v>-100.494269</v>
       </c>
       <c r="C62">
         <v>48.190050999999997</v>
       </c>
       <c r="D62" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E62">
         <v>2</v>
       </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F62">
+        <f t="shared" si="0"/>
+        <v>-99.994269000000003</v>
+      </c>
+      <c r="G62">
+        <v>16</v>
+      </c>
+      <c r="H62">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>32</v>
       </c>
       <c r="B63">
-        <v>-83.947596000000004</v>
+        <v>-83.447596000000004</v>
       </c>
       <c r="C63">
         <v>41.152164999999997</v>
       </c>
       <c r="D63" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E63">
         <v>2</v>
       </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F63">
+        <f t="shared" si="0"/>
+        <v>-82.947596000000004</v>
+      </c>
+      <c r="G63">
+        <v>16</v>
+      </c>
+      <c r="H63">
+        <v>2.0750000000000002</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>33</v>
       </c>
       <c r="B64">
-        <v>-98.284328000000002</v>
+        <v>-97.784328000000002</v>
       </c>
       <c r="C64">
         <v>36.331032999999998</v>
       </c>
       <c r="D64" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E64">
         <v>0</v>
       </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F64">
+        <f t="shared" si="0"/>
+        <v>-97.284328000000002</v>
+      </c>
+      <c r="G64">
+        <v>16</v>
+      </c>
+      <c r="H64">
+        <v>-6.1159999999999997</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>33</v>
       </c>
       <c r="B65">
-        <v>-98.284328000000002</v>
+        <v>-97.784328000000002</v>
       </c>
       <c r="C65">
         <v>36.331032999999998</v>
       </c>
       <c r="D65" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E65">
         <v>1</v>
       </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F65">
+        <f t="shared" si="0"/>
+        <v>-97.284328000000002</v>
+      </c>
+      <c r="G65">
+        <v>16</v>
+      </c>
+      <c r="H65">
+        <v>-6.1159999999999997</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>34</v>
       </c>
       <c r="B66">
-        <v>-121.52998700000001</v>
+        <v>-121.02998700000001</v>
       </c>
       <c r="C66">
         <v>44.804492000000003</v>
       </c>
       <c r="D66" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E66">
         <v>0</v>
       </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F66">
+        <f t="shared" si="0"/>
+        <v>-120.52998700000001</v>
+      </c>
+      <c r="G66">
+        <v>16</v>
+      </c>
+      <c r="H66">
+        <v>-5.9509999999999996</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>34</v>
       </c>
       <c r="B67">
-        <v>-121.52998700000001</v>
+        <v>-121.02998700000001</v>
       </c>
       <c r="C67">
         <v>44.804492000000003</v>
       </c>
       <c r="D67" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E67">
         <v>1</v>
       </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F67">
+        <f t="shared" ref="F67:F87" si="1">B67+0.5</f>
+        <v>-120.52998700000001</v>
+      </c>
+      <c r="G67">
+        <v>16</v>
+      </c>
+      <c r="H67">
+        <v>-5.9509999999999996</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>34</v>
       </c>
       <c r="B68">
-        <v>-119.963954</v>
+        <v>-119.463954</v>
       </c>
       <c r="C68">
         <v>43.170872000000003</v>
       </c>
       <c r="D68" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E68">
         <v>2</v>
       </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F68">
+        <f t="shared" si="1"/>
+        <v>-118.963954</v>
+      </c>
+      <c r="G68">
+        <v>16</v>
+      </c>
+      <c r="H68">
+        <v>-1.258</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>35</v>
       </c>
       <c r="B69">
-        <v>-78.881307000000007</v>
+        <v>-77.381307000000007</v>
       </c>
       <c r="C69">
-        <v>41.538652999999996</v>
+        <v>41.288652999999996</v>
       </c>
       <c r="D69" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E69">
         <v>0</v>
       </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F69">
+        <f t="shared" si="1"/>
+        <v>-76.881307000000007</v>
+      </c>
+      <c r="G69">
+        <v>16</v>
+      </c>
+      <c r="H69">
+        <v>8.4269999999999996</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>35</v>
       </c>
       <c r="B70">
-        <v>-78.881307000000007</v>
+        <v>-77.381307000000007</v>
       </c>
       <c r="C70">
-        <v>41.538652999999996</v>
+        <v>41.288652999999996</v>
       </c>
       <c r="D70" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E70">
         <v>1</v>
       </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F70">
+        <f t="shared" si="1"/>
+        <v>-76.881307000000007</v>
+      </c>
+      <c r="G70">
+        <v>16</v>
+      </c>
+      <c r="H70">
+        <v>8.4269999999999996</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>35</v>
       </c>
       <c r="B71">
-        <v>-78.383743999999993</v>
+        <v>-77.883743999999993</v>
       </c>
       <c r="C71">
         <v>40.342810999999998</v>
       </c>
       <c r="D71" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E71">
         <v>2</v>
       </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F71">
+        <f t="shared" si="1"/>
+        <v>-77.383743999999993</v>
+      </c>
+      <c r="G71">
+        <v>16</v>
+      </c>
+      <c r="H71">
+        <v>8.4269999999999996</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>36</v>
       </c>
       <c r="B72">
-        <v>-82.191519999999997</v>
+        <v>-81.691519999999997</v>
       </c>
       <c r="C72">
         <v>34.694054000000001</v>
       </c>
       <c r="D72" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E72">
         <v>2</v>
       </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F72">
+        <f t="shared" si="1"/>
+        <v>-81.191519999999997</v>
+      </c>
+      <c r="G72">
+        <v>16</v>
+      </c>
+      <c r="H72">
+        <v>10.048999999999999</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>36</v>
       </c>
       <c r="B73">
-        <v>-80.712255999999996</v>
+        <v>-80.951887999999997</v>
       </c>
       <c r="C73">
-        <v>33.041580000000003</v>
+        <v>32.791580000000003</v>
       </c>
       <c r="D73" t="s">
         <v>54</v>
@@ -1945,50 +2988,80 @@
       <c r="E73">
         <v>1</v>
       </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F73">
+        <f t="shared" si="1"/>
+        <v>-80.451887999999997</v>
+      </c>
+      <c r="G73">
+        <v>16</v>
+      </c>
+      <c r="H73">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>37</v>
       </c>
       <c r="B74">
-        <v>-101.962514</v>
+        <v>-101.462514</v>
       </c>
       <c r="C74">
         <v>45.278523</v>
       </c>
       <c r="D74" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E74">
         <v>2</v>
       </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F74">
+        <f t="shared" si="1"/>
+        <v>-100.962514</v>
+      </c>
+      <c r="G74">
+        <v>16</v>
+      </c>
+      <c r="H74">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>38</v>
       </c>
       <c r="B75">
-        <v>-88.926848000000007</v>
+        <v>-88.426848000000007</v>
       </c>
       <c r="C75">
         <v>35.760626000000002</v>
       </c>
       <c r="D75" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E75">
         <v>2</v>
       </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F75">
+        <f t="shared" si="1"/>
+        <v>-87.926848000000007</v>
+      </c>
+      <c r="G75">
+        <v>16</v>
+      </c>
+      <c r="H75">
+        <v>2.6030000000000002</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>38</v>
       </c>
       <c r="B76">
-        <v>-84.403547000000003</v>
+        <v>-84.153547000000003</v>
       </c>
       <c r="C76">
-        <v>36.199865000000003</v>
+        <v>35.699865000000003</v>
       </c>
       <c r="D76" t="s">
         <v>54</v>
@@ -1996,81 +3069,131 @@
       <c r="E76">
         <v>1</v>
       </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F76">
+        <f t="shared" si="1"/>
+        <v>-83.653547000000003</v>
+      </c>
+      <c r="G76">
+        <v>16</v>
+      </c>
+      <c r="H76">
+        <v>2.6030000000000002</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>39</v>
       </c>
       <c r="B77">
-        <v>-100.89321200000001</v>
+        <v>-99.393212000000005</v>
       </c>
       <c r="C77">
-        <v>33.598441000000001</v>
+        <v>32.598441000000001</v>
       </c>
       <c r="D77" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E77">
         <v>0</v>
       </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F77">
+        <f t="shared" si="1"/>
+        <v>-98.893212000000005</v>
+      </c>
+      <c r="G77">
+        <v>16</v>
+      </c>
+      <c r="H77">
+        <v>-5.5389999999999997</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>39</v>
       </c>
       <c r="B78">
-        <v>-100.89321200000001</v>
+        <v>-99.393212000000005</v>
       </c>
       <c r="C78">
-        <v>33.598441000000001</v>
+        <v>32.598441000000001</v>
       </c>
       <c r="D78" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E78">
         <v>1</v>
       </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F78">
+        <f t="shared" si="1"/>
+        <v>-98.893212000000005</v>
+      </c>
+      <c r="G78">
+        <v>16</v>
+      </c>
+      <c r="H78">
+        <v>-5.5389999999999997</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>40</v>
       </c>
       <c r="B79">
-        <v>-78.542058999999995</v>
+        <v>-78.042058999999995</v>
       </c>
       <c r="C79">
         <v>38.490935999999998</v>
       </c>
       <c r="D79" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E79">
         <v>0</v>
       </c>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F79">
+        <f t="shared" si="1"/>
+        <v>-77.542058999999995</v>
+      </c>
+      <c r="G79">
+        <v>16</v>
+      </c>
+      <c r="H79">
+        <v>8.6310000000000002</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>40</v>
       </c>
       <c r="B80">
-        <v>-78.542058999999995</v>
+        <v>-78.042058999999995</v>
       </c>
       <c r="C80">
         <v>38.490935999999998</v>
       </c>
       <c r="D80" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E80">
         <v>1</v>
       </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F80">
+        <f t="shared" si="1"/>
+        <v>-77.542058999999995</v>
+      </c>
+      <c r="G80">
+        <v>16</v>
+      </c>
+      <c r="H80">
+        <v>8.6310000000000002</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>40</v>
       </c>
       <c r="B81">
-        <v>-78.067111999999995</v>
+        <v>-77.567111999999995</v>
       </c>
       <c r="C81">
         <v>37.886555999999999</v>
@@ -2081,111 +3204,730 @@
       <c r="E81">
         <v>1</v>
       </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F81">
+        <f t="shared" si="1"/>
+        <v>-77.067111999999995</v>
+      </c>
+      <c r="G81">
+        <v>16</v>
+      </c>
+      <c r="H81">
+        <v>8.6310000000000002</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>41</v>
       </c>
       <c r="B82">
-        <v>-119.963954</v>
+        <v>-119.463954</v>
       </c>
       <c r="C82">
         <v>48.198455000000003</v>
       </c>
       <c r="D82" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E82">
         <v>2</v>
       </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F82">
+        <f t="shared" si="1"/>
+        <v>-118.963954</v>
+      </c>
+      <c r="G82">
+        <v>16</v>
+      </c>
+      <c r="H82">
+        <v>-1.1379999999999999</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>42</v>
       </c>
       <c r="B83">
-        <v>-80.713243000000006</v>
+        <v>-80.213243000000006</v>
       </c>
       <c r="C83">
         <v>39.107841000000001</v>
       </c>
       <c r="D83" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E83">
         <v>2</v>
       </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F83">
+        <f t="shared" si="1"/>
+        <v>-79.713243000000006</v>
+      </c>
+      <c r="G83">
+        <v>16</v>
+      </c>
+      <c r="H83">
+        <v>7.9509999999999996</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>43</v>
       </c>
       <c r="B84">
-        <v>-91.08887</v>
+        <v>-90.58887</v>
       </c>
       <c r="C84">
         <v>45.401415999999998</v>
       </c>
       <c r="D84" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E84">
         <v>0</v>
       </c>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F84">
+        <f t="shared" si="1"/>
+        <v>-90.08887</v>
+      </c>
+      <c r="G84">
+        <v>12</v>
+      </c>
+      <c r="H84">
+        <v>7.66</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>43</v>
       </c>
       <c r="B85">
-        <v>-91.08887</v>
+        <v>-90.58887</v>
       </c>
       <c r="C85">
         <v>45.401415999999998</v>
       </c>
       <c r="D85" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E85">
         <v>1</v>
       </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F85">
+        <f t="shared" si="1"/>
+        <v>-90.08887</v>
+      </c>
+      <c r="G85">
+        <v>12</v>
+      </c>
+      <c r="H85">
+        <v>7.66</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>43</v>
       </c>
       <c r="B86">
-        <v>-89.777112000000002</v>
+        <v>-89.527112000000002</v>
       </c>
       <c r="C86">
-        <v>44.002977999999999</v>
+        <v>43.752977999999999</v>
       </c>
       <c r="D86" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E86">
         <v>2</v>
       </c>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F86">
+        <f t="shared" si="1"/>
+        <v>-89.027112000000002</v>
+      </c>
+      <c r="G86">
+        <v>12</v>
+      </c>
+      <c r="H86">
+        <v>4.5830000000000002</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>44</v>
       </c>
       <c r="B87">
-        <v>-108.740233</v>
+        <v>-108.240233</v>
       </c>
       <c r="C87">
         <v>44.093012000000002</v>
       </c>
       <c r="D87" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E87">
         <v>2</v>
+      </c>
+      <c r="F87">
+        <f t="shared" si="1"/>
+        <v>-107.740233</v>
+      </c>
+      <c r="G87">
+        <v>16</v>
+      </c>
+      <c r="H87">
+        <v>-9.3239999999999998</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77F38634-F1CC-4ED7-BA51-69AEBE411EAA}">
+  <dimension ref="A1:C49"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>217</v>
+      </c>
+      <c r="B1" t="s">
+        <v>218</v>
+      </c>
+      <c r="C1" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C2">
+        <v>3.7120000000000002</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B3" t="s">
+        <v>124</v>
+      </c>
+      <c r="C3">
+        <v>-9.5419999999999998</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>125</v>
+      </c>
+      <c r="B4" t="s">
+        <v>126</v>
+      </c>
+      <c r="C4">
+        <v>1.6080000000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>127</v>
+      </c>
+      <c r="B5" t="s">
+        <v>128</v>
+      </c>
+      <c r="C5">
+        <v>-13.988</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>129</v>
+      </c>
+      <c r="B6" t="s">
+        <v>130</v>
+      </c>
+      <c r="C6">
+        <v>-5.7110000000000003</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>131</v>
+      </c>
+      <c r="B7" t="s">
+        <v>132</v>
+      </c>
+      <c r="C7">
+        <v>15.811</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>133</v>
+      </c>
+      <c r="B8" t="s">
+        <v>134</v>
+      </c>
+      <c r="C8">
+        <v>13.367000000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>135</v>
+      </c>
+      <c r="B9" t="s">
+        <v>136</v>
+      </c>
+      <c r="C9">
+        <v>4.3109999999999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>137</v>
+      </c>
+      <c r="B10" t="s">
+        <v>138</v>
+      </c>
+      <c r="C10">
+        <v>9.6660000000000004</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>139</v>
+      </c>
+      <c r="B11" t="s">
+        <v>140</v>
+      </c>
+      <c r="C11">
+        <v>-11.868</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>141</v>
+      </c>
+      <c r="B12" t="s">
+        <v>142</v>
+      </c>
+      <c r="C12">
+        <v>5.819</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>143</v>
+      </c>
+      <c r="B13" t="s">
+        <v>144</v>
+      </c>
+      <c r="C13">
+        <v>7.7939999999999996</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>145</v>
+      </c>
+      <c r="B14" t="s">
+        <v>146</v>
+      </c>
+      <c r="C14">
+        <v>1.9330000000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>147</v>
+      </c>
+      <c r="B15" t="s">
+        <v>148</v>
+      </c>
+      <c r="C15">
+        <v>-2.4580000000000002</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>149</v>
+      </c>
+      <c r="B16" t="s">
+        <v>150</v>
+      </c>
+      <c r="C16">
+        <v>6.5060000000000002</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>151</v>
+      </c>
+      <c r="B17" t="s">
+        <v>152</v>
+      </c>
+      <c r="C17">
+        <v>3.8730000000000002</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>153</v>
+      </c>
+      <c r="B18" t="s">
+        <v>154</v>
+      </c>
+      <c r="C18">
+        <v>15.035</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>155</v>
+      </c>
+      <c r="B19" t="s">
+        <v>156</v>
+      </c>
+      <c r="C19">
+        <v>11.31</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>157</v>
+      </c>
+      <c r="B20" t="s">
+        <v>158</v>
+      </c>
+      <c r="C20">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>159</v>
+      </c>
+      <c r="B21" t="s">
+        <v>160</v>
+      </c>
+      <c r="C21">
+        <v>6.34</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>161</v>
+      </c>
+      <c r="B22" t="s">
+        <v>162</v>
+      </c>
+      <c r="C22">
+        <v>1.1930000000000001</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>163</v>
+      </c>
+      <c r="B23" t="s">
+        <v>164</v>
+      </c>
+      <c r="C23">
+        <v>1.7430000000000001</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>165</v>
+      </c>
+      <c r="B24" t="s">
+        <v>166</v>
+      </c>
+      <c r="C24">
+        <v>2.3279999999999998</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>167</v>
+      </c>
+      <c r="B25" t="s">
+        <v>168</v>
+      </c>
+      <c r="C25">
+        <v>-10.62</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>169</v>
+      </c>
+      <c r="B26" t="s">
+        <v>170</v>
+      </c>
+      <c r="C26">
+        <v>-2.0270000000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>171</v>
+      </c>
+      <c r="B27" t="s">
+        <v>172</v>
+      </c>
+      <c r="C27">
+        <v>-13.016</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>173</v>
+      </c>
+      <c r="B28" t="s">
+        <v>174</v>
+      </c>
+      <c r="C28">
+        <v>16.097999999999999</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>175</v>
+      </c>
+      <c r="B29" t="s">
+        <v>176</v>
+      </c>
+      <c r="C29">
+        <v>12.529</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>177</v>
+      </c>
+      <c r="B30" t="s">
+        <v>178</v>
+      </c>
+      <c r="C30">
+        <v>-5.7110000000000003</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>179</v>
+      </c>
+      <c r="B31" t="s">
+        <v>180</v>
+      </c>
+      <c r="C31">
+        <v>11.925000000000001</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>181</v>
+      </c>
+      <c r="B32" t="s">
+        <v>182</v>
+      </c>
+      <c r="C32">
+        <v>10.353</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>183</v>
+      </c>
+      <c r="B33" t="s">
+        <v>184</v>
+      </c>
+      <c r="C33">
+        <v>-3.327</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>185</v>
+      </c>
+      <c r="B34" t="s">
+        <v>186</v>
+      </c>
+      <c r="C34">
+        <v>8.8130000000000006</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>187</v>
+      </c>
+      <c r="B35" t="s">
+        <v>188</v>
+      </c>
+      <c r="C35">
+        <v>0.46</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>189</v>
+      </c>
+      <c r="B36" t="s">
+        <v>190</v>
+      </c>
+      <c r="C36">
+        <v>-16.538</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>191</v>
+      </c>
+      <c r="B37" t="s">
+        <v>192</v>
+      </c>
+      <c r="C37">
+        <v>12.481999999999999</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>193</v>
+      </c>
+      <c r="B38" t="s">
+        <v>194</v>
+      </c>
+      <c r="C38">
+        <v>16.504000000000001</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>195</v>
+      </c>
+      <c r="B39" t="s">
+        <v>196</v>
+      </c>
+      <c r="C39">
+        <v>7.1580000000000004</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>197</v>
+      </c>
+      <c r="B40" t="s">
+        <v>198</v>
+      </c>
+      <c r="C40">
+        <v>-3.7989999999999999</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>199</v>
+      </c>
+      <c r="B41" t="s">
+        <v>200</v>
+      </c>
+      <c r="C41">
+        <v>4.4249999999999998</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>201</v>
+      </c>
+      <c r="B42" t="s">
+        <v>202</v>
+      </c>
+      <c r="C42">
+        <v>-4.2830000000000004</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>203</v>
+      </c>
+      <c r="B43" t="s">
+        <v>204</v>
+      </c>
+      <c r="C43">
+        <v>-8.5690000000000008</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>205</v>
+      </c>
+      <c r="B44" t="s">
+        <v>206</v>
+      </c>
+      <c r="C44">
+        <v>16.645</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B45" t="s">
+        <v>208</v>
+      </c>
+      <c r="C45">
+        <v>8.1760000000000002</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>209</v>
+      </c>
+      <c r="B46" t="s">
+        <v>210</v>
+      </c>
+      <c r="C46">
+        <v>-15.874000000000001</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>211</v>
+      </c>
+      <c r="B47" t="s">
+        <v>212</v>
+      </c>
+      <c r="C47">
+        <v>8.5169999999999995</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>213</v>
+      </c>
+      <c r="B48" t="s">
+        <v>214</v>
+      </c>
+      <c r="C48">
+        <v>4.7389999999999999</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>215</v>
+      </c>
+      <c r="B49" t="s">
+        <v>216</v>
+      </c>
+      <c r="C49">
+        <v>-8.7690000000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Finished Red Record Map Recreation
</commit_message>
<xml_diff>
--- a/Slow Reveal Recreations/anti-lynching-bill-map/text_position.xlsx
+++ b/Slow Reveal Recreations/anti-lynching-bill-map/text_position.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gvsu365-my.sharepoint.com/personal/s_cousilou_gvsu_edu/Documents/GVSU/Work/R Files/slow-reveal-graphs/Slow Reveal Recreations/anti-lynching-bill-map/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1445" documentId="11_F25DC773A252ABDACC10485159997CA65BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE15901E-103B-4B5A-9D37-824BF914DB3D}"/>
+  <xr:revisionPtr revIDLastSave="1470" documentId="11_F25DC773A252ABDACC10485159997CA65BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37D436DB-6254-4CA5-8963-FEAC4C651CD0}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Horizontal Text" sheetId="1" r:id="rId1"/>
@@ -345,54 +345,9 @@
     <t>display_step</t>
   </si>
   <si>
-    <t>&lt;span style='color:red;'&gt;292&lt;/span&gt;&lt;span style='color:#FCF2DA;'&gt; -&lt;/span&gt;</t>
-  </si>
-  <si>
-    <t>&lt;span style='color:red;'&gt;8&lt;/span&gt;&lt;span style='color:#FCF2DA;'&gt; - 1&lt;/span&gt;</t>
-  </si>
-  <si>
-    <t>&lt;span style='color:red;'&gt;29&lt;/span&gt;&lt;span style='color:#FCF2DA;'&gt; - 5&lt;/span&gt;</t>
-  </si>
-  <si>
-    <t>&lt;span style='color:red;'&gt;201&lt;/span&gt;&lt;span style='color:#FCF2DA;'&gt; -&lt;/span&gt;</t>
-  </si>
-  <si>
-    <t>&lt;span style='color:red;'&gt;429&lt;/span&gt;&lt;span style='color:#FCF2DA;'&gt; -&lt;/span&gt;</t>
-  </si>
-  <si>
-    <t>&lt;span style='color:red;'&gt;11&lt;/span&gt;&lt;span style='color:#FCF2DA;'&gt; - 1&lt;/span&gt;</t>
-  </si>
-  <si>
-    <t>&lt;span style='color:red;'&gt;171&lt;/span&gt;&lt;span style='color:#FCF2DA;'&gt; -&lt;/span&gt;</t>
-  </si>
-  <si>
-    <t>&lt;span style='color:red;'&gt;1&lt;/span&gt;&lt;span style='color:#FCF2DA;'&gt; - 1&lt;/span&gt;</t>
-  </si>
-  <si>
-    <t>&lt;span style='color:red;'&gt;17&lt;/span&gt;&lt;span style='color:#FCF2DA;'&gt; - 2&lt;/span&gt;</t>
-  </si>
-  <si>
-    <t>&lt;span style='color:red;'&gt;4&lt;/span&gt;&lt;span style='color:#FCF2DA;'&gt; - 1&lt;/span&gt;</t>
-  </si>
-  <si>
-    <t>&lt;span style='color:red;'&gt;84&lt;/span&gt;&lt;span style='color:#FCF2DA;'&gt; - 1&lt;/span&gt;</t>
-  </si>
-  <si>
-    <t>&lt;span style='color:red;'&gt;99&lt;/span&gt;&lt;span style='color:#FCF2DA;'&gt; - 5&lt;/span&gt;</t>
-  </si>
-  <si>
-    <t>&lt;span style='color:red;'&gt;354&lt;/span&gt;&lt;span style='color:#FCF2DA;'&gt; - 15&lt;/span&gt;</t>
-  </si>
-  <si>
-    <t>&lt;span style='color:red;'&gt;80&lt;/span&gt;&lt;span style='color:#FCF2DA;'&gt; -&lt;/span&gt;</t>
-  </si>
-  <si>
     <t>x_adj</t>
   </si>
   <si>
-    <t>&lt;span style='color:red;'&gt;405&lt;/span&gt;&lt;span style='color:#FCF2DA;'&gt; -&lt;/span&gt;</t>
-  </si>
-  <si>
     <t>&lt;span style='color:red;'&gt;405&lt;/span&gt;&lt;span style='color:black;'&gt; -&lt;/span&gt;</t>
   </si>
   <si>
@@ -697,6 +652,51 @@
   </si>
   <si>
     <t>angle</t>
+  </si>
+  <si>
+    <t>&lt;span style='color:red;'&gt;292&lt;/span&gt;&lt;span style='color:#F8EAD1;'&gt; -&lt;/span&gt;</t>
+  </si>
+  <si>
+    <t>&lt;span style='color:red;'&gt;8&lt;/span&gt;&lt;span style='color:#F8EAD1;'&gt; - 1&lt;/span&gt;</t>
+  </si>
+  <si>
+    <t>&lt;span style='color:red;'&gt;29&lt;/span&gt;&lt;span style='color:#F8EAD1;'&gt; - 5&lt;/span&gt;</t>
+  </si>
+  <si>
+    <t>&lt;span style='color:red;'&gt;201&lt;/span&gt;&lt;span style='color:#F8EAD1;'&gt; -&lt;/span&gt;</t>
+  </si>
+  <si>
+    <t>&lt;span style='color:red;'&gt;429&lt;/span&gt;&lt;span style='color:#F8EAD1;'&gt; -&lt;/span&gt;</t>
+  </si>
+  <si>
+    <t>&lt;span style='color:red;'&gt;11&lt;/span&gt;&lt;span style='color:#F8EAD1;'&gt; - 1&lt;/span&gt;</t>
+  </si>
+  <si>
+    <t>&lt;span style='color:red;'&gt;171&lt;/span&gt;&lt;span style='color:#F8EAD1;'&gt; -&lt;/span&gt;</t>
+  </si>
+  <si>
+    <t>&lt;span style='color:red;'&gt;1&lt;/span&gt;&lt;span style='color:#F8EAD1;'&gt; - 1&lt;/span&gt;</t>
+  </si>
+  <si>
+    <t>&lt;span style='color:red;'&gt;17&lt;/span&gt;&lt;span style='color:#F8EAD1;'&gt; - 2&lt;/span&gt;</t>
+  </si>
+  <si>
+    <t>&lt;span style='color:red;'&gt;4&lt;/span&gt;&lt;span style='color:#F8EAD1;'&gt; - 1&lt;/span&gt;</t>
+  </si>
+  <si>
+    <t>&lt;span style='color:red;'&gt;405&lt;/span&gt;&lt;span style='color:#F8EAD1;'&gt; -&lt;/span&gt;</t>
+  </si>
+  <si>
+    <t>&lt;span style='color:red;'&gt;84&lt;/span&gt;&lt;span style='color:#F8EAD1;'&gt; - 1&lt;/span&gt;</t>
+  </si>
+  <si>
+    <t>&lt;span style='color:red;'&gt;99&lt;/span&gt;&lt;span style='color:#F8EAD1;'&gt; - 5&lt;/span&gt;</t>
+  </si>
+  <si>
+    <t>&lt;span style='color:red;'&gt;354&lt;/span&gt;&lt;span style='color:#F8EAD1;'&gt; - 15&lt;/span&gt;</t>
+  </si>
+  <si>
+    <t>&lt;span style='color:red;'&gt;80&lt;/span&gt;&lt;span style='color:#F8EAD1;'&gt; -&lt;/span&gt;</t>
   </si>
 </sst>
 </file>
@@ -1043,13 +1043,13 @@
         <v>101</v>
       </c>
       <c r="F1" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="G1" t="s">
-        <v>119</v>
+        <v>104</v>
       </c>
       <c r="H1" t="s">
-        <v>219</v>
+        <v>204</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1063,7 +1063,7 @@
         <v>34.217106000000001</v>
       </c>
       <c r="D2" t="s">
-        <v>102</v>
+        <v>205</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1144,7 +1144,7 @@
         <v>36.310676999999998</v>
       </c>
       <c r="D5" t="s">
-        <v>103</v>
+        <v>206</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -1228,7 +1228,7 @@
         <v>53</v>
       </c>
       <c r="E8">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F8">
         <f t="shared" si="0"/>
@@ -1279,7 +1279,7 @@
         <v>40.873595999999999</v>
       </c>
       <c r="D10" t="s">
-        <v>104</v>
+        <v>207</v>
       </c>
       <c r="E10">
         <v>0</v>
@@ -1471,7 +1471,7 @@
         <v>60</v>
       </c>
       <c r="E17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F17">
         <f t="shared" si="0"/>
@@ -1495,7 +1495,7 @@
         <v>29.882432999999999</v>
       </c>
       <c r="D18" t="s">
-        <v>105</v>
+        <v>208</v>
       </c>
       <c r="E18">
         <v>0</v>
@@ -1576,7 +1576,7 @@
         <v>34.283602000000002</v>
       </c>
       <c r="D21" t="s">
-        <v>106</v>
+        <v>209</v>
       </c>
       <c r="E21">
         <v>0</v>
@@ -1657,7 +1657,7 @@
         <v>44.787768999999997</v>
       </c>
       <c r="D24" t="s">
-        <v>107</v>
+        <v>210</v>
       </c>
       <c r="E24">
         <v>0</v>
@@ -1741,7 +1741,7 @@
         <v>64</v>
       </c>
       <c r="E27">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F27">
         <f t="shared" si="0"/>
@@ -1768,7 +1768,7 @@
         <v>70</v>
       </c>
       <c r="E28">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F28">
         <f t="shared" si="0"/>
@@ -1795,7 +1795,7 @@
         <v>65</v>
       </c>
       <c r="E29">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F29">
         <f t="shared" si="0"/>
@@ -1822,7 +1822,7 @@
         <v>64</v>
       </c>
       <c r="E30">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F30">
         <f t="shared" si="0"/>
@@ -1846,7 +1846,7 @@
         <v>38.002592999999997</v>
       </c>
       <c r="D31" t="s">
-        <v>108</v>
+        <v>211</v>
       </c>
       <c r="E31">
         <v>0</v>
@@ -1927,10 +1927,10 @@
         <v>32.215719999999997</v>
       </c>
       <c r="D34" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="E34">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F34">
         <f t="shared" si="0"/>
@@ -1981,7 +1981,7 @@
         <v>46.504477000000001</v>
       </c>
       <c r="D36" t="s">
-        <v>109</v>
+        <v>212</v>
       </c>
       <c r="E36">
         <v>0</v>
@@ -2062,7 +2062,7 @@
         <v>39.130082999999999</v>
       </c>
       <c r="D39" t="s">
-        <v>110</v>
+        <v>213</v>
       </c>
       <c r="E39">
         <v>0</v>
@@ -2146,7 +2146,7 @@
         <v>44.375965000000001</v>
       </c>
       <c r="D42" t="s">
-        <v>111</v>
+        <v>214</v>
       </c>
       <c r="E42">
         <v>0</v>
@@ -2230,7 +2230,7 @@
         <v>73</v>
       </c>
       <c r="E45">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F45">
         <f t="shared" si="0"/>
@@ -2254,7 +2254,7 @@
         <v>34.194929000000002</v>
       </c>
       <c r="D46" t="s">
-        <v>117</v>
+        <v>215</v>
       </c>
       <c r="E46">
         <v>0</v>
@@ -2281,7 +2281,7 @@
         <v>34.194929000000002</v>
       </c>
       <c r="D47" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="E47">
         <v>1</v>
@@ -2335,7 +2335,7 @@
         <v>39.841631999999997</v>
       </c>
       <c r="D49" t="s">
-        <v>112</v>
+        <v>216</v>
       </c>
       <c r="E49">
         <v>0</v>
@@ -2419,7 +2419,7 @@
         <v>80</v>
       </c>
       <c r="E52">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F52">
         <f t="shared" si="0"/>
@@ -2446,7 +2446,7 @@
         <v>81</v>
       </c>
       <c r="E53">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F53">
         <f t="shared" si="0"/>
@@ -2473,7 +2473,7 @@
         <v>82</v>
       </c>
       <c r="E54">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F54">
         <f t="shared" si="0"/>
@@ -2554,7 +2554,7 @@
         <v>84</v>
       </c>
       <c r="E57">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F57">
         <f t="shared" si="0"/>
@@ -2581,7 +2581,7 @@
         <v>85</v>
       </c>
       <c r="E58">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F58">
         <f t="shared" si="0"/>
@@ -2608,7 +2608,7 @@
         <v>86</v>
       </c>
       <c r="E59">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F59">
         <f t="shared" si="0"/>
@@ -2662,7 +2662,7 @@
         <v>88</v>
       </c>
       <c r="E61">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F61">
         <f t="shared" si="0"/>
@@ -2689,7 +2689,7 @@
         <v>89</v>
       </c>
       <c r="E62">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F62">
         <f t="shared" si="0"/>
@@ -2716,7 +2716,7 @@
         <v>85</v>
       </c>
       <c r="E63">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F63">
         <f t="shared" si="0"/>
@@ -2740,7 +2740,7 @@
         <v>36.331032999999998</v>
       </c>
       <c r="D64" t="s">
-        <v>113</v>
+        <v>217</v>
       </c>
       <c r="E64">
         <v>0</v>
@@ -2794,7 +2794,7 @@
         <v>44.804492000000003</v>
       </c>
       <c r="D66" t="s">
-        <v>111</v>
+        <v>214</v>
       </c>
       <c r="E66">
         <v>0</v>
@@ -2875,7 +2875,7 @@
         <v>41.288652999999996</v>
       </c>
       <c r="D69" t="s">
-        <v>111</v>
+        <v>214</v>
       </c>
       <c r="E69">
         <v>0</v>
@@ -2959,7 +2959,7 @@
         <v>93</v>
       </c>
       <c r="E72">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F72">
         <f t="shared" si="1"/>
@@ -3013,7 +3013,7 @@
         <v>85</v>
       </c>
       <c r="E74">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F74">
         <f t="shared" si="1"/>
@@ -3040,7 +3040,7 @@
         <v>94</v>
       </c>
       <c r="E75">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F75">
         <f t="shared" si="1"/>
@@ -3091,7 +3091,7 @@
         <v>32.598441000000001</v>
       </c>
       <c r="D77" t="s">
-        <v>114</v>
+        <v>218</v>
       </c>
       <c r="E77">
         <v>0</v>
@@ -3145,7 +3145,7 @@
         <v>38.490935999999998</v>
       </c>
       <c r="D79" t="s">
-        <v>115</v>
+        <v>219</v>
       </c>
       <c r="E79">
         <v>0</v>
@@ -3229,7 +3229,7 @@
         <v>95</v>
       </c>
       <c r="E82">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F82">
         <f t="shared" si="1"/>
@@ -3256,7 +3256,7 @@
         <v>96</v>
       </c>
       <c r="E83">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F83">
         <f t="shared" si="1"/>
@@ -3280,7 +3280,7 @@
         <v>45.401415999999998</v>
       </c>
       <c r="D84" t="s">
-        <v>111</v>
+        <v>214</v>
       </c>
       <c r="E84">
         <v>0</v>
@@ -3364,7 +3364,7 @@
         <v>98</v>
       </c>
       <c r="E87">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F87">
         <f t="shared" si="1"/>
@@ -3390,21 +3390,21 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>217</v>
+        <v>202</v>
       </c>
       <c r="B1" t="s">
-        <v>218</v>
+        <v>203</v>
       </c>
       <c r="C1" t="s">
-        <v>219</v>
+        <v>204</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>121</v>
+        <v>106</v>
       </c>
       <c r="B2" t="s">
-        <v>122</v>
+        <v>107</v>
       </c>
       <c r="C2">
         <v>3.7120000000000002</v>
@@ -3412,10 +3412,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>123</v>
+        <v>108</v>
       </c>
       <c r="B3" t="s">
-        <v>124</v>
+        <v>109</v>
       </c>
       <c r="C3">
         <v>-9.5419999999999998</v>
@@ -3423,10 +3423,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>125</v>
+        <v>110</v>
       </c>
       <c r="B4" t="s">
-        <v>126</v>
+        <v>111</v>
       </c>
       <c r="C4">
         <v>1.6080000000000001</v>
@@ -3434,10 +3434,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>127</v>
+        <v>112</v>
       </c>
       <c r="B5" t="s">
-        <v>128</v>
+        <v>113</v>
       </c>
       <c r="C5">
         <v>-13.988</v>
@@ -3445,10 +3445,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>129</v>
+        <v>114</v>
       </c>
       <c r="B6" t="s">
-        <v>130</v>
+        <v>115</v>
       </c>
       <c r="C6">
         <v>-5.7110000000000003</v>
@@ -3456,10 +3456,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="B7" t="s">
-        <v>132</v>
+        <v>117</v>
       </c>
       <c r="C7">
         <v>15.811</v>
@@ -3467,10 +3467,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>133</v>
+        <v>118</v>
       </c>
       <c r="B8" t="s">
-        <v>134</v>
+        <v>119</v>
       </c>
       <c r="C8">
         <v>13.367000000000001</v>
@@ -3478,10 +3478,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>135</v>
+        <v>120</v>
       </c>
       <c r="B9" t="s">
-        <v>136</v>
+        <v>121</v>
       </c>
       <c r="C9">
         <v>4.3109999999999999</v>
@@ -3489,10 +3489,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>137</v>
+        <v>122</v>
       </c>
       <c r="B10" t="s">
-        <v>138</v>
+        <v>123</v>
       </c>
       <c r="C10">
         <v>9.6660000000000004</v>
@@ -3500,10 +3500,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>139</v>
+        <v>124</v>
       </c>
       <c r="B11" t="s">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="C11">
         <v>-11.868</v>
@@ -3511,10 +3511,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>141</v>
+        <v>126</v>
       </c>
       <c r="B12" t="s">
-        <v>142</v>
+        <v>127</v>
       </c>
       <c r="C12">
         <v>5.819</v>
@@ -3522,10 +3522,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>143</v>
+        <v>128</v>
       </c>
       <c r="B13" t="s">
-        <v>144</v>
+        <v>129</v>
       </c>
       <c r="C13">
         <v>7.7939999999999996</v>
@@ -3533,10 +3533,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>145</v>
+        <v>130</v>
       </c>
       <c r="B14" t="s">
-        <v>146</v>
+        <v>131</v>
       </c>
       <c r="C14">
         <v>1.9330000000000001</v>
@@ -3544,10 +3544,10 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>147</v>
+        <v>132</v>
       </c>
       <c r="B15" t="s">
-        <v>148</v>
+        <v>133</v>
       </c>
       <c r="C15">
         <v>-2.4580000000000002</v>
@@ -3555,10 +3555,10 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>149</v>
+        <v>134</v>
       </c>
       <c r="B16" t="s">
-        <v>150</v>
+        <v>135</v>
       </c>
       <c r="C16">
         <v>6.5060000000000002</v>
@@ -3566,10 +3566,10 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>151</v>
+        <v>136</v>
       </c>
       <c r="B17" t="s">
-        <v>152</v>
+        <v>137</v>
       </c>
       <c r="C17">
         <v>3.8730000000000002</v>
@@ -3577,10 +3577,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>153</v>
+        <v>138</v>
       </c>
       <c r="B18" t="s">
-        <v>154</v>
+        <v>139</v>
       </c>
       <c r="C18">
         <v>15.035</v>
@@ -3588,10 +3588,10 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>155</v>
+        <v>140</v>
       </c>
       <c r="B19" t="s">
-        <v>156</v>
+        <v>141</v>
       </c>
       <c r="C19">
         <v>11.31</v>
@@ -3599,10 +3599,10 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>157</v>
+        <v>142</v>
       </c>
       <c r="B20" t="s">
-        <v>158</v>
+        <v>143</v>
       </c>
       <c r="C20">
         <v>16</v>
@@ -3610,10 +3610,10 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>159</v>
+        <v>144</v>
       </c>
       <c r="B21" t="s">
-        <v>160</v>
+        <v>145</v>
       </c>
       <c r="C21">
         <v>6.34</v>
@@ -3621,10 +3621,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>161</v>
+        <v>146</v>
       </c>
       <c r="B22" t="s">
-        <v>162</v>
+        <v>147</v>
       </c>
       <c r="C22">
         <v>1.1930000000000001</v>
@@ -3632,10 +3632,10 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>163</v>
+        <v>148</v>
       </c>
       <c r="B23" t="s">
-        <v>164</v>
+        <v>149</v>
       </c>
       <c r="C23">
         <v>1.7430000000000001</v>
@@ -3643,10 +3643,10 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>165</v>
+        <v>150</v>
       </c>
       <c r="B24" t="s">
-        <v>166</v>
+        <v>151</v>
       </c>
       <c r="C24">
         <v>2.3279999999999998</v>
@@ -3654,10 +3654,10 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>167</v>
+        <v>152</v>
       </c>
       <c r="B25" t="s">
-        <v>168</v>
+        <v>153</v>
       </c>
       <c r="C25">
         <v>-10.62</v>
@@ -3665,10 +3665,10 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>169</v>
+        <v>154</v>
       </c>
       <c r="B26" t="s">
-        <v>170</v>
+        <v>155</v>
       </c>
       <c r="C26">
         <v>-2.0270000000000001</v>
@@ -3676,10 +3676,10 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>171</v>
+        <v>156</v>
       </c>
       <c r="B27" t="s">
-        <v>172</v>
+        <v>157</v>
       </c>
       <c r="C27">
         <v>-13.016</v>
@@ -3687,10 +3687,10 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>173</v>
+        <v>158</v>
       </c>
       <c r="B28" t="s">
-        <v>174</v>
+        <v>159</v>
       </c>
       <c r="C28">
         <v>16.097999999999999</v>
@@ -3698,10 +3698,10 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>175</v>
+        <v>160</v>
       </c>
       <c r="B29" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C29">
         <v>12.529</v>
@@ -3709,10 +3709,10 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>177</v>
+        <v>162</v>
       </c>
       <c r="B30" t="s">
-        <v>178</v>
+        <v>163</v>
       </c>
       <c r="C30">
         <v>-5.7110000000000003</v>
@@ -3720,10 +3720,10 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>179</v>
+        <v>164</v>
       </c>
       <c r="B31" t="s">
-        <v>180</v>
+        <v>165</v>
       </c>
       <c r="C31">
         <v>11.925000000000001</v>
@@ -3731,10 +3731,10 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>181</v>
+        <v>166</v>
       </c>
       <c r="B32" t="s">
-        <v>182</v>
+        <v>167</v>
       </c>
       <c r="C32">
         <v>10.353</v>
@@ -3742,10 +3742,10 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>183</v>
+        <v>168</v>
       </c>
       <c r="B33" t="s">
-        <v>184</v>
+        <v>169</v>
       </c>
       <c r="C33">
         <v>-3.327</v>
@@ -3753,10 +3753,10 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>185</v>
+        <v>170</v>
       </c>
       <c r="B34" t="s">
-        <v>186</v>
+        <v>171</v>
       </c>
       <c r="C34">
         <v>8.8130000000000006</v>
@@ -3764,10 +3764,10 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>187</v>
+        <v>172</v>
       </c>
       <c r="B35" t="s">
-        <v>188</v>
+        <v>173</v>
       </c>
       <c r="C35">
         <v>0.46</v>
@@ -3775,10 +3775,10 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>189</v>
+        <v>174</v>
       </c>
       <c r="B36" t="s">
-        <v>190</v>
+        <v>175</v>
       </c>
       <c r="C36">
         <v>-16.538</v>
@@ -3786,10 +3786,10 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>191</v>
+        <v>176</v>
       </c>
       <c r="B37" t="s">
-        <v>192</v>
+        <v>177</v>
       </c>
       <c r="C37">
         <v>12.481999999999999</v>
@@ -3797,10 +3797,10 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>193</v>
+        <v>178</v>
       </c>
       <c r="B38" t="s">
-        <v>194</v>
+        <v>179</v>
       </c>
       <c r="C38">
         <v>16.504000000000001</v>
@@ -3808,10 +3808,10 @@
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>195</v>
+        <v>180</v>
       </c>
       <c r="B39" t="s">
-        <v>196</v>
+        <v>181</v>
       </c>
       <c r="C39">
         <v>7.1580000000000004</v>
@@ -3819,10 +3819,10 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>197</v>
+        <v>182</v>
       </c>
       <c r="B40" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="C40">
         <v>-3.7989999999999999</v>
@@ -3830,10 +3830,10 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>199</v>
+        <v>184</v>
       </c>
       <c r="B41" t="s">
-        <v>200</v>
+        <v>185</v>
       </c>
       <c r="C41">
         <v>4.4249999999999998</v>
@@ -3841,10 +3841,10 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>201</v>
+        <v>186</v>
       </c>
       <c r="B42" t="s">
-        <v>202</v>
+        <v>187</v>
       </c>
       <c r="C42">
         <v>-4.2830000000000004</v>
@@ -3852,10 +3852,10 @@
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>203</v>
+        <v>188</v>
       </c>
       <c r="B43" t="s">
-        <v>204</v>
+        <v>189</v>
       </c>
       <c r="C43">
         <v>-8.5690000000000008</v>
@@ -3863,10 +3863,10 @@
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="B44" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="C44">
         <v>16.645</v>
@@ -3874,10 +3874,10 @@
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>207</v>
+        <v>192</v>
       </c>
       <c r="B45" t="s">
-        <v>208</v>
+        <v>193</v>
       </c>
       <c r="C45">
         <v>8.1760000000000002</v>
@@ -3885,10 +3885,10 @@
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>209</v>
+        <v>194</v>
       </c>
       <c r="B46" t="s">
-        <v>210</v>
+        <v>195</v>
       </c>
       <c r="C46">
         <v>-15.874000000000001</v>
@@ -3896,10 +3896,10 @@
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>211</v>
+        <v>196</v>
       </c>
       <c r="B47" t="s">
-        <v>212</v>
+        <v>197</v>
       </c>
       <c r="C47">
         <v>8.5169999999999995</v>
@@ -3907,10 +3907,10 @@
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>213</v>
+        <v>198</v>
       </c>
       <c r="B48" t="s">
-        <v>214</v>
+        <v>199</v>
       </c>
       <c r="C48">
         <v>4.7389999999999999</v>
@@ -3918,10 +3918,10 @@
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>215</v>
+        <v>200</v>
       </c>
       <c r="B49" t="s">
-        <v>216</v>
+        <v>201</v>
       </c>
       <c r="C49">
         <v>-8.7690000000000001</v>

</xml_diff>